<commit_message>
Opps duplicadas: con el criterio de Monica (proyecto + subvencion = una opp; dos opps si hay mucho tiempo o, sobre todo, portales distintos), Excel de lo que queda: lo que se hace, dudas con su criterio y las dos-opps para repasar (20-oct)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/opps/opps_duplicadas_en_seco.xlsx
+++ b/docs/opps/opps_duplicadas_en_seco.xlsx
@@ -6422,7 +6422,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>DAN-2016-212</t>
+          <t>DAN-2016-209</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>MADRID/1APROVINCIA/GETAFE/travesiadecastro2</t>
+          <t>MADRID/1APROVINCIA/GETAFE/castro2</t>
         </is>
       </c>
       <c r="K50" t="inlineStr"/>
@@ -6485,7 +6485,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>DAN-2016-209</t>
+          <t>DAN-2016-212</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -6521,7 +6521,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>MADRID/1APROVINCIA/GETAFE/castro2</t>
+          <t>MADRID/1APROVINCIA/GETAFE/travesiadecastro2</t>
         </is>
       </c>
       <c r="K51" t="inlineStr"/>
@@ -6686,7 +6686,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>DAN-2023-160</t>
+          <t>DAN-2023-159</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -6722,7 +6722,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>MADRID/1APROVINCIA/SAN SEBASTIAN DE LOS REYES/travesiasanonofre7</t>
+          <t>MADRID/sanonofre7</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -6736,7 +6736,7 @@
         <v>0</v>
       </c>
       <c r="O54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P54" t="n">
         <v>0</v>
@@ -6753,7 +6753,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>DAN-2023-159</t>
+          <t>DAN-2023-160</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -6789,7 +6789,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>MADRID/sanonofre7</t>
+          <t>MADRID/1APROVINCIA/SAN SEBASTIAN DE LOS REYES/travesiasanonofre7</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -6803,7 +6803,7 @@
         <v>0</v>
       </c>
       <c r="O55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P55" t="n">
         <v>0</v>
@@ -7340,12 +7340,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ALV-2026-005</t>
+          <t>DAN-2026-024</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Principes de España 17 y 19, Coslada (avenida)</t>
+          <t>Principes de España 19, Coslada (avenida)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -7360,7 +7360,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Alvaro</t>
+          <t>Daniel</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -7371,26 +7371,26 @@
       <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr">
         <is>
-          <t>PRINCIPES DE ESPAÑA 17 esc. 1; PRINCIPES DE ESPAÑA 19 esc. 1</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr"/>
+          <t>PRINCIPES DE ESPAÑA 19 esc. 1</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>MADRID/1APROVINCIA/COSLADA/avlosprincipesdeespaña19</t>
+        </is>
+      </c>
       <c r="K64" t="inlineStr">
         <is>
           <t>Ascensor, doble embarque con derribo de escalera</t>
         </is>
       </c>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>HE-2026-0021 enviada_comunidad: Ascensor, Subvenciones; HE-2026-0022 devuelta_firmada firmada 2026-04-06: Accesibilidad, Rampa</t>
-        </is>
-      </c>
+      <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr"/>
       <c r="N64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O64" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="P64" t="n">
         <v>0</v>
@@ -7407,12 +7407,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>DAN-2026-024</t>
+          <t>ALV-2026-005</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Principes de España 19, Coslada (avenida)</t>
+          <t>Principes de España 17 y 19, Coslada (avenida)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -7427,7 +7427,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Daniel</t>
+          <t>Alvaro</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -7438,26 +7438,26 @@
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr">
         <is>
-          <t>PRINCIPES DE ESPAÑA 19 esc. 1</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>MADRID/1APROVINCIA/COSLADA/avlosprincipesdeespaña19</t>
-        </is>
-      </c>
+          <t>PRINCIPES DE ESPAÑA 17 esc. 1; PRINCIPES DE ESPAÑA 19 esc. 1</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr"/>
       <c r="K65" t="inlineStr">
         <is>
           <t>Ascensor, doble embarque con derribo de escalera</t>
         </is>
       </c>
-      <c r="L65" t="inlineStr"/>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>HE-2026-0021 enviada_comunidad: Ascensor, Subvenciones; HE-2026-0022 devuelta_firmada firmada 2026-04-06: Accesibilidad, Rampa</t>
+        </is>
+      </c>
       <c r="M65" t="inlineStr"/>
       <c r="N65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O65" t="n">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="P65" t="n">
         <v>0</v>
@@ -7943,12 +7943,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>DAN-2026-084</t>
+          <t>DAN-2026-086</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Salamanca 1, 3, 5 y 7 + Del Empecinado 23, Mostoles</t>
+          <t>Salamanca 5, Mostoles</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -7968,13 +7968,17 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>CP SALAMANCA 1-3-5-7 Y EMPECINADO 23 MOSTOLES</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr"/>
+          <t>CP SALAMANCA 5 MOSTOLES</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>H80681042</t>
+        </is>
+      </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>EMPECINADO DEL 23; SALAMANCA 1; SALAMANCA 3; SALAMANCA 5; SALAMANCA 7</t>
+          <t>SALAMANCA 5</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -7985,7 +7989,7 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>HE-2026-0172 devuelta_firmada firmada 2026-05-11: 3 Presupuestos/Arreglo cubierta</t>
+          <t>HE-2026-0174 devuelta_firmada firmada 2026-05-11: 3 Presupuestos/Arreglo cubierta</t>
         </is>
       </c>
       <c r="M73" t="inlineStr"/>
@@ -8081,12 +8085,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>DAN-2026-086</t>
+          <t>DAN-2026-084</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Salamanca 5, Mostoles</t>
+          <t>Salamanca 1, 3, 5 y 7 + Del Empecinado 23, Mostoles</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8106,17 +8110,13 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>CP SALAMANCA 5 MOSTOLES</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>H80681042</t>
-        </is>
-      </c>
+          <t>CP SALAMANCA 1-3-5-7 Y EMPECINADO 23 MOSTOLES</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr">
         <is>
-          <t>SALAMANCA 5</t>
+          <t>EMPECINADO DEL 23; SALAMANCA 1; SALAMANCA 3; SALAMANCA 5; SALAMANCA 7</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -8127,7 +8127,7 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>HE-2026-0174 devuelta_firmada firmada 2026-05-11: 3 Presupuestos/Arreglo cubierta</t>
+          <t>HE-2026-0172 devuelta_firmada firmada 2026-05-11: 3 Presupuestos/Arreglo cubierta</t>
         </is>
       </c>
       <c r="M75" t="inlineStr"/>

</xml_diff>